<commit_message>
Refactor - add sublineage layer
</commit_message>
<xml_diff>
--- a/tabular/reference/herv_sublineage_data.xlsx
+++ b/tabular/reference/herv_sublineage_data.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C24C156-F07E-B645-A2F4-C48A75F7E4E6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D532016-7CAC-6B4A-89F9-868901BFD1CD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2320" yWindow="500" windowWidth="27120" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1680" yWindow="520" windowWidth="27120" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sublineage" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="229">
   <si>
     <t>sequenceID</t>
   </si>
@@ -635,6 +636,78 @@
   </si>
   <si>
     <t>Standardised lineage name</t>
+  </si>
+  <si>
+    <t>HERV-Fc1</t>
+  </si>
+  <si>
+    <t>ERV-1.HF.Fc.1</t>
+  </si>
+  <si>
+    <t>lineage</t>
+  </si>
+  <si>
+    <t>AncRecon</t>
+  </si>
+  <si>
+    <t>HERV-Fc2</t>
+  </si>
+  <si>
+    <t>ERV-1.HF.Fc.2</t>
+  </si>
+  <si>
+    <t>human endogenous retrovirus F(c) 2</t>
+  </si>
+  <si>
+    <t>human endogenous retrovirus F(c) 1</t>
+  </si>
+  <si>
+    <t>HERV-T1</t>
+  </si>
+  <si>
+    <t>ERV-1.Gamma.T1</t>
+  </si>
+  <si>
+    <t>human endogenous retrovirus T1</t>
+  </si>
+  <si>
+    <t>HERV-T2</t>
+  </si>
+  <si>
+    <t>ERV-1.Gamma.T2</t>
+  </si>
+  <si>
+    <t>human endogenous retrovirus T2</t>
+  </si>
+  <si>
+    <t>HERVT1</t>
+  </si>
+  <si>
+    <t>HERVT2</t>
+  </si>
+  <si>
+    <t>HERV-T3</t>
+  </si>
+  <si>
+    <t>ERV-1.Gamma.T3</t>
+  </si>
+  <si>
+    <t>human endogenous retrovirus T3</t>
+  </si>
+  <si>
+    <t>HERVT3</t>
+  </si>
+  <si>
+    <t>HERVT</t>
+  </si>
+  <si>
+    <t>RRHERV-I</t>
+  </si>
+  <si>
+    <t>Retinoic acid-responsive human endogenous retrovirus I</t>
+  </si>
+  <si>
+    <t>ERV-1.Gamma.I</t>
   </si>
 </sst>
 </file>
@@ -1526,13 +1599,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB9083D8-DE01-F14E-ACB5-AF33867092C5}">
-  <dimension ref="A1:U57"/>
+  <dimension ref="A1:U58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.33203125" customWidth="1"/>
     <col min="2" max="2" width="27.5" customWidth="1"/>
     <col min="3" max="3" width="18.5" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
+    <col min="4" max="4" width="50.1640625" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="11" max="11" width="21" customWidth="1"/>
   </cols>
@@ -4832,6 +4905,67 @@
         <v>3</v>
       </c>
     </row>
+    <row r="58" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A58" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H58" s="2">
+        <v>9464</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L58" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="M58" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="N58" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="O58" s="2">
+        <v>7</v>
+      </c>
+      <c r="P58" s="2"/>
+      <c r="Q58" s="2"/>
+      <c r="R58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T58" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="U58" s="2">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T57">
     <sortCondition ref="I2:I57"/>
@@ -4839,7 +4973,67 @@
     <sortCondition ref="L2:L57"/>
     <sortCondition ref="C2:C57"/>
   </sortState>
-  <conditionalFormatting sqref="U58:U1048576 U1:U48">
+  <conditionalFormatting sqref="U63:U1048576 U1:U48">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U49:U52">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U53:U54">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U55">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U56">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U57">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -4851,55 +5045,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U49:U52">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U53:U54">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U55">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U56">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U57">
+  <conditionalFormatting sqref="U58">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -4913,4 +5059,426 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF64240C-8748-834A-9B04-2536247ED9D0}">
+  <dimension ref="A1:U6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="O4" s="2">
+        <v>7</v>
+      </c>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="2">
+        <v>7</v>
+      </c>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U5" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="O6" s="2">
+        <v>7</v>
+      </c>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U6" s="2">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="U2">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U4">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U3">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U5">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U6">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U1">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor - moved HERV sublineages and fragments from ERVdb lineage layer
</commit_message>
<xml_diff>
--- a/tabular/reference/herv_sublineage_data.xlsx
+++ b/tabular/reference/herv_sublineage_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D532016-7CAC-6B4A-89F9-868901BFD1CD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05097530-0173-0D4A-A691-99FA59B25F84}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1680" yWindow="520" windowWidth="27120" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="999" uniqueCount="233">
   <si>
     <t>sequenceID</t>
   </si>
@@ -708,6 +708,18 @@
   </si>
   <si>
     <t>ERV-1.Gamma.I</t>
+  </si>
+  <si>
+    <t>Iotaretrovirus</t>
+  </si>
+  <si>
+    <t>HERV-ADP</t>
+  </si>
+  <si>
+    <t>human endogenous retrovirus ADP</t>
+  </si>
+  <si>
+    <t>ERV-1.Iota.ADP</t>
   </si>
 </sst>
 </file>
@@ -1599,7 +1611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB9083D8-DE01-F14E-ACB5-AF33867092C5}">
-  <dimension ref="A1:U58"/>
+  <dimension ref="A1:U59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.33203125" customWidth="1"/>
@@ -1793,28 +1805,28 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>45</v>
+        <v>226</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>172</v>
+        <v>228</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>108</v>
+        <v>226</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>227</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>45</v>
+        <v>226</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H4" s="2">
-        <v>4936</v>
+        <v>9464</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>24</v>
@@ -1823,55 +1835,59 @@
         <v>5</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="L4" s="1"/>
+        <v>25</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>225</v>
+      </c>
       <c r="M4" s="2" t="s">
         <v>6</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O4" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="O4" s="2">
+        <v>7</v>
+      </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="2" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="T4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="U4" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>47</v>
+        <v>230</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>173</v>
+        <v>232</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>109</v>
+        <v>230</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>231</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>143</v>
+        <v>207</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>47</v>
+        <v>230</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H5" s="2">
-        <v>9084</v>
+        <v>7590</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>24</v>
@@ -1880,53 +1896,57 @@
         <v>5</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>44</v>
+        <v>229</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O5" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="O5" s="2">
+        <v>1</v>
+      </c>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="U5" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E6" s="2"/>
+        <v>108</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>147</v>
+      </c>
       <c r="F6" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H6" s="2">
-        <v>8439</v>
+        <v>4936</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>24</v>
@@ -1939,14 +1959,12 @@
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="2" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="O6" s="2">
-        <v>1</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="O6" s="2"/>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="2" t="s">
@@ -1964,28 +1982,28 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>143</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H7" s="2">
-        <v>7613</v>
+        <v>9084</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>24</v>
@@ -1994,7 +2012,7 @@
         <v>5</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="2" t="s">
@@ -2007,7 +2025,7 @@
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="S7" s="2" t="s">
         <v>13</v>
@@ -2016,33 +2034,31 @@
         <v>13</v>
       </c>
       <c r="U7" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>147</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H8" s="2">
-        <v>1786</v>
+        <v>8439</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>24</v>
@@ -2051,16 +2067,18 @@
         <v>5</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O8" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="O8" s="2">
+        <v>1</v>
+      </c>
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
       <c r="R8" s="2" t="s">
@@ -2078,28 +2096,28 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>143</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H9" s="2">
-        <v>9161</v>
+        <v>7613</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>24</v>
@@ -2112,14 +2130,12 @@
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="2" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="O9" s="2">
-        <v>1</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="O9" s="2"/>
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
       <c r="R9" s="2" t="s">
@@ -2132,31 +2148,33 @@
         <v>13</v>
       </c>
       <c r="U9" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>147</v>
+      </c>
       <c r="F10" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H10" s="2">
-        <v>8120</v>
+        <v>1786</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>24</v>
@@ -2192,28 +2210,28 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>113</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H11" s="2">
-        <v>4060</v>
+        <v>9161</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>24</v>
@@ -2226,16 +2244,18 @@
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O11" s="2"/>
+        <v>23</v>
+      </c>
+      <c r="O11" s="2">
+        <v>1</v>
+      </c>
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
       <c r="R11" s="2" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="S11" s="2" t="s">
         <v>13</v>
@@ -2244,33 +2264,31 @@
         <v>13</v>
       </c>
       <c r="U11" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>147</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H12" s="2">
-        <v>4798</v>
+        <v>8120</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>24</v>
@@ -2306,28 +2324,28 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>124</v>
+        <v>56</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H13" s="2">
-        <v>6639</v>
+        <v>4060</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>24</v>
@@ -2363,28 +2381,28 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>125</v>
+        <v>57</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>147</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H14" s="2">
-        <v>933</v>
+        <v>4798</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>24</v>
@@ -2420,28 +2438,28 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H15" s="2">
-        <v>4936</v>
+        <v>6639</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>24</v>
@@ -2477,28 +2495,28 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>147</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H16" s="2">
-        <v>5356</v>
+        <v>933</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>24</v>
@@ -2534,28 +2552,28 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>185</v>
+        <v>60</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>183</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>147</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H17" s="2">
-        <v>6387</v>
+        <v>4936</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>24</v>
@@ -2591,28 +2609,28 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>186</v>
+        <v>61</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>184</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>147</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H18" s="2">
-        <v>6758</v>
+        <v>5356</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>24</v>
@@ -2648,28 +2666,28 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H19" s="2">
-        <v>5217</v>
+        <v>6387</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>24</v>
@@ -2705,28 +2723,28 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H20" s="2">
-        <v>4871</v>
+        <v>6758</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>24</v>
@@ -2751,7 +2769,7 @@
         <v>46</v>
       </c>
       <c r="S20" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T20" s="2" t="s">
         <v>13</v>
@@ -2762,28 +2780,28 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H21" s="2">
-        <v>7048</v>
+        <v>5217</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>24</v>
@@ -2819,28 +2837,28 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>190</v>
+        <v>65</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>188</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>67</v>
+        <v>131</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>143</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H22" s="2">
-        <v>4102</v>
+        <v>4871</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>24</v>
@@ -2862,7 +2880,7 @@
       <c r="P22" s="2"/>
       <c r="Q22" s="2"/>
       <c r="R22" s="2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="S22" s="2" t="s">
         <v>12</v>
@@ -2871,33 +2889,33 @@
         <v>13</v>
       </c>
       <c r="U22" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:21" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>191</v>
+        <v>66</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>189</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>147</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H23" s="2">
-        <v>4981</v>
+        <v>7048</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>24</v>
@@ -2906,11 +2924,9 @@
         <v>5</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>69</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="L23" s="1"/>
       <c r="M23" s="2" t="s">
         <v>6</v>
       </c>
@@ -2921,7 +2937,7 @@
       <c r="P23" s="2"/>
       <c r="Q23" s="2"/>
       <c r="R23" s="2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="S23" s="2" t="s">
         <v>13</v>
@@ -2930,33 +2946,33 @@
         <v>13</v>
       </c>
       <c r="U23" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>116</v>
+        <v>67</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>143</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H24" s="2">
-        <v>6996</v>
+        <v>4102</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>24</v>
@@ -2965,11 +2981,9 @@
         <v>5</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="L24" s="1" t="s">
-        <v>71</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="L24" s="1"/>
       <c r="M24" s="2" t="s">
         <v>6</v>
       </c>
@@ -2983,7 +2997,7 @@
         <v>12</v>
       </c>
       <c r="S24" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="T24" s="2" t="s">
         <v>13</v>
@@ -2994,28 +3008,28 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>74</v>
+        <v>138</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H25" s="2">
-        <v>11027</v>
+        <v>4981</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>24</v>
@@ -3027,7 +3041,7 @@
         <v>68</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M25" s="2" t="s">
         <v>6</v>
@@ -3039,7 +3053,7 @@
       <c r="P25" s="2"/>
       <c r="Q25" s="2"/>
       <c r="R25" s="2" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="S25" s="2" t="s">
         <v>13</v>
@@ -3048,33 +3062,33 @@
         <v>13</v>
       </c>
       <c r="U25" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>116</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H26" s="2">
-        <v>8987</v>
+        <v>6996</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>24</v>
@@ -3098,7 +3112,7 @@
       <c r="P26" s="2"/>
       <c r="Q26" s="2"/>
       <c r="R26" s="2" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="S26" s="2" t="s">
         <v>13</v>
@@ -3107,33 +3121,33 @@
         <v>13</v>
       </c>
       <c r="U26" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H27" s="2">
-        <v>7418</v>
+        <v>11027</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>24</v>
@@ -3157,7 +3171,7 @@
       <c r="P27" s="2"/>
       <c r="Q27" s="2"/>
       <c r="R27" s="2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="S27" s="2" t="s">
         <v>13</v>
@@ -3166,33 +3180,33 @@
         <v>13</v>
       </c>
       <c r="U27" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>114</v>
+        <v>75</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H28" s="2">
-        <v>5586</v>
+        <v>8987</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>24</v>
@@ -3203,7 +3217,9 @@
       <c r="K28" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="L28" s="1"/>
+      <c r="L28" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="M28" s="2" t="s">
         <v>6</v>
       </c>
@@ -3228,28 +3244,28 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H29" s="2">
-        <v>6918</v>
+        <v>7418</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>24</v>
@@ -3260,7 +3276,9 @@
       <c r="K29" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="L29" s="1"/>
+      <c r="L29" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="M29" s="2" t="s">
         <v>6</v>
       </c>
@@ -3271,7 +3289,7 @@
       <c r="P29" s="2"/>
       <c r="Q29" s="2"/>
       <c r="R29" s="2" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="S29" s="2" t="s">
         <v>13</v>
@@ -3280,33 +3298,33 @@
         <v>13</v>
       </c>
       <c r="U29" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>198</v>
+        <v>70</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>196</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H30" s="2">
-        <v>3944</v>
+        <v>5586</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>24</v>
@@ -3342,26 +3360,28 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>199</v>
+        <v>72</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>197</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="E31" s="2"/>
+        <v>115</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>145</v>
+      </c>
       <c r="F31" s="2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H31" s="2">
-        <v>7133</v>
+        <v>6918</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>24</v>
@@ -3397,28 +3417,28 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>147</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H32" s="2">
-        <v>4285</v>
+        <v>3944</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>24</v>
@@ -3454,28 +3474,26 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>147</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H33" s="2">
-        <v>4880</v>
+        <v>7133</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>24</v>
@@ -3511,28 +3529,28 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>147</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H34" s="2">
-        <v>2880</v>
+        <v>4285</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>24</v>
@@ -3554,42 +3572,42 @@
       <c r="P34" s="2"/>
       <c r="Q34" s="2"/>
       <c r="R34" s="2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="S34" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T34" s="2" t="s">
         <v>13</v>
       </c>
       <c r="U34" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>203</v>
+        <v>81</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>201</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>83</v>
+        <v>136</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>147</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H35" s="2">
-        <v>8665</v>
+        <v>4880</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>24</v>
@@ -3611,7 +3629,7 @@
       <c r="P35" s="2"/>
       <c r="Q35" s="2"/>
       <c r="R35" s="2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="S35" s="2" t="s">
         <v>13</v>
@@ -3620,46 +3638,44 @@
         <v>13</v>
       </c>
       <c r="U35" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>150</v>
+        <v>82</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>202</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>106</v>
+        <v>137</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>100</v>
+        <v>147</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H36" s="2">
-        <v>7048</v>
+        <v>2880</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>5</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="L36" s="1" t="s">
-        <v>10</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="L36" s="1"/>
       <c r="M36" s="2" t="s">
         <v>6</v>
       </c>
@@ -3673,61 +3689,57 @@
         <v>12</v>
       </c>
       <c r="S36" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="T36" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U36" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>151</v>
+        <v>203</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>100</v>
+        <v>147</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H37" s="2">
-        <v>6364</v>
+        <v>8665</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>5</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="L37" s="1" t="s">
-        <v>10</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="L37" s="1"/>
       <c r="M37" s="2" t="s">
         <v>6</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="O37" s="2">
-        <v>7</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="O37" s="2"/>
       <c r="P37" s="2"/>
       <c r="Q37" s="2"/>
       <c r="R37" s="2" t="s">
@@ -3737,21 +3749,21 @@
         <v>13</v>
       </c>
       <c r="T37" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U37" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>106</v>
@@ -3766,7 +3778,7 @@
         <v>3</v>
       </c>
       <c r="H38" s="2">
-        <v>9472</v>
+        <v>7048</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>4</v>
@@ -3784,18 +3796,16 @@
         <v>6</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="O38" s="2">
-        <v>47</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="O38" s="2"/>
       <c r="P38" s="2"/>
       <c r="Q38" s="2"/>
       <c r="R38" s="2" t="s">
         <v>12</v>
       </c>
       <c r="S38" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="T38" s="2" t="s">
         <v>12</v>
@@ -3806,13 +3816,13 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>106</v>
@@ -3827,7 +3837,7 @@
         <v>3</v>
       </c>
       <c r="H39" s="2">
-        <v>7045</v>
+        <v>6364</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>4</v>
@@ -3845,9 +3855,11 @@
         <v>6</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O39" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="O39" s="2">
+        <v>7</v>
+      </c>
       <c r="P39" s="2"/>
       <c r="Q39" s="2"/>
       <c r="R39" s="2" t="s">
@@ -3865,13 +3877,13 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>106</v>
@@ -3886,7 +3898,7 @@
         <v>3</v>
       </c>
       <c r="H40" s="2">
-        <v>10243</v>
+        <v>9472</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>4</v>
@@ -3907,7 +3919,7 @@
         <v>7</v>
       </c>
       <c r="O40" s="2">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="P40" s="2"/>
       <c r="Q40" s="2"/>
@@ -3915,7 +3927,7 @@
         <v>12</v>
       </c>
       <c r="S40" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="T40" s="2" t="s">
         <v>12</v>
@@ -3926,13 +3938,13 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>106</v>
@@ -3947,7 +3959,7 @@
         <v>3</v>
       </c>
       <c r="H41" s="2">
-        <v>8355</v>
+        <v>7045</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>4</v>
@@ -3965,11 +3977,9 @@
         <v>6</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="O41" s="2">
-        <v>25</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="O41" s="2"/>
       <c r="P41" s="2"/>
       <c r="Q41" s="2"/>
       <c r="R41" s="2" t="s">
@@ -3987,13 +3997,13 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>106</v>
@@ -4008,7 +4018,7 @@
         <v>3</v>
       </c>
       <c r="H42" s="2">
-        <v>7274</v>
+        <v>10243</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>4</v>
@@ -4029,7 +4039,7 @@
         <v>7</v>
       </c>
       <c r="O42" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="P42" s="2"/>
       <c r="Q42" s="2"/>
@@ -4037,7 +4047,7 @@
         <v>12</v>
       </c>
       <c r="S42" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="T42" s="2" t="s">
         <v>12</v>
@@ -4048,13 +4058,13 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>106</v>
@@ -4069,7 +4079,7 @@
         <v>3</v>
       </c>
       <c r="H43" s="2">
-        <v>8214</v>
+        <v>8355</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>4</v>
@@ -4090,7 +4100,7 @@
         <v>7</v>
       </c>
       <c r="O43" s="2">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="P43" s="2"/>
       <c r="Q43" s="2"/>
@@ -4109,46 +4119,50 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F44" s="2" t="s">
-        <v>30</v>
+      <c r="F44" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H44" s="2">
-        <v>6070</v>
+        <v>7274</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>5</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="L44" s="1"/>
+        <v>9</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="M44" s="2" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O44" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="O44" s="2">
+        <v>10</v>
+      </c>
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
       <c r="R44" s="2" t="s">
@@ -4158,54 +4172,58 @@
         <v>13</v>
       </c>
       <c r="T44" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="U44" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>31</v>
+        <v>143</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H45" s="2">
-        <v>5667</v>
+        <v>8214</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="J45" s="2" t="s">
         <v>5</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="L45" s="1"/>
+        <v>9</v>
+      </c>
+      <c r="L45" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="M45" s="2" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O45" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="O45" s="2">
+        <v>104</v>
+      </c>
       <c r="P45" s="2"/>
       <c r="Q45" s="2"/>
       <c r="R45" s="2" t="s">
@@ -4215,36 +4233,36 @@
         <v>13</v>
       </c>
       <c r="T45" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="U45" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>104</v>
+        <v>30</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>143</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H46" s="2">
-        <v>5714</v>
+        <v>6070</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>28</v>
@@ -4280,22 +4298,22 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>103</v>
+        <v>31</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>101</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>3</v>
@@ -4337,28 +4355,28 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>117</v>
+        <v>32</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H48" s="2">
-        <v>4996</v>
+        <v>5714</v>
       </c>
       <c r="I48" s="2" t="s">
         <v>28</v>
@@ -4394,28 +4412,28 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>118</v>
+        <v>33</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H49" s="2">
-        <v>3556</v>
+        <v>5667</v>
       </c>
       <c r="I49" s="2" t="s">
         <v>28</v>
@@ -4437,7 +4455,7 @@
       <c r="P49" s="2"/>
       <c r="Q49" s="2"/>
       <c r="R49" s="2" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="S49" s="2" t="s">
         <v>13</v>
@@ -4446,33 +4464,33 @@
         <v>13</v>
       </c>
       <c r="U49" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H50" s="2">
-        <v>5343</v>
+        <v>4996</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>28</v>
@@ -4494,7 +4512,7 @@
       <c r="P50" s="2"/>
       <c r="Q50" s="2"/>
       <c r="R50" s="2" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="S50" s="2" t="s">
         <v>13</v>
@@ -4503,33 +4521,33 @@
         <v>13</v>
       </c>
       <c r="U50" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H51" s="2">
-        <v>5530</v>
+        <v>3556</v>
       </c>
       <c r="I51" s="2" t="s">
         <v>28</v>
@@ -4551,7 +4569,7 @@
       <c r="P51" s="2"/>
       <c r="Q51" s="2"/>
       <c r="R51" s="2" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="S51" s="2" t="s">
         <v>13</v>
@@ -4565,28 +4583,28 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H52" s="2">
-        <v>3329</v>
+        <v>5343</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>28</v>
@@ -4622,28 +4640,28 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H53" s="2">
-        <v>3037</v>
+        <v>5530</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>28</v>
@@ -4665,7 +4683,7 @@
       <c r="P53" s="2"/>
       <c r="Q53" s="2"/>
       <c r="R53" s="2" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="S53" s="2" t="s">
         <v>13</v>
@@ -4679,28 +4697,28 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A54" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H54" s="2">
-        <v>5685</v>
+        <v>3329</v>
       </c>
       <c r="I54" s="2" t="s">
         <v>28</v>
@@ -4722,7 +4740,7 @@
       <c r="P54" s="2"/>
       <c r="Q54" s="2"/>
       <c r="R54" s="2" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="S54" s="2" t="s">
         <v>13</v>
@@ -4736,28 +4754,28 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A55" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>147</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H55" s="2">
-        <v>5023</v>
+        <v>3037</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>28</v>
@@ -4779,7 +4797,7 @@
       <c r="P55" s="2"/>
       <c r="Q55" s="2"/>
       <c r="R55" s="2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="S55" s="2" t="s">
         <v>13</v>
@@ -4788,33 +4806,33 @@
         <v>13</v>
       </c>
       <c r="U55" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A56" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>143</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H56" s="2">
-        <v>6189</v>
+        <v>5685</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>28</v>
@@ -4850,28 +4868,28 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A57" s="5" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>102</v>
+        <v>139</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H57" s="2">
-        <v>5246</v>
+        <v>5023</v>
       </c>
       <c r="I57" s="2" t="s">
         <v>28</v>
@@ -4880,7 +4898,7 @@
         <v>5</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="L57" s="1"/>
       <c r="M57" s="2" t="s">
@@ -4907,73 +4925,138 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A58" s="5" t="s">
-        <v>226</v>
+        <v>43</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>228</v>
+        <v>169</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>226</v>
+        <v>43</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>227</v>
+        <v>140</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>143</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>226</v>
+        <v>43</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>3</v>
       </c>
       <c r="H58" s="2">
-        <v>9464</v>
+        <v>6189</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="J58" s="2" t="s">
         <v>5</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L58" s="1" t="s">
-        <v>225</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="L58" s="1"/>
       <c r="M58" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="O58" s="2">
-        <v>7</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="O58" s="2"/>
       <c r="P58" s="2"/>
       <c r="Q58" s="2"/>
       <c r="R58" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="S58" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="T58" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="U58" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A59" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H59" s="2">
+        <v>5246</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="L59" s="1"/>
+      <c r="M59" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O59" s="2"/>
+      <c r="P59" s="2"/>
+      <c r="Q59" s="2"/>
+      <c r="R59" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S58" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T58" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="U58" s="2">
-        <v>2</v>
+      <c r="S59" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="T59" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="U59" s="2">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T57">
-    <sortCondition ref="I2:I57"/>
-    <sortCondition ref="K2:K57"/>
-    <sortCondition ref="L2:L57"/>
-    <sortCondition ref="C2:C57"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U59">
+    <sortCondition ref="I2:I59"/>
+    <sortCondition ref="K2:K59"/>
+    <sortCondition ref="L2:L59"/>
+    <sortCondition ref="C2:C59"/>
   </sortState>
   <conditionalFormatting sqref="U63:U1048576 U1:U48">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U49:U52">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -4985,7 +5068,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U49:U52">
+  <conditionalFormatting sqref="U53:U54">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -4997,7 +5080,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U53:U54">
+  <conditionalFormatting sqref="U55">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -5009,7 +5092,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U55">
+  <conditionalFormatting sqref="U56">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -5021,7 +5104,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U56">
+  <conditionalFormatting sqref="U57">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -5033,8 +5116,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U57">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="U58">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5045,7 +5128,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U58">
+  <conditionalFormatting sqref="U59">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
Import legacy alias mappings for ERV loci
</commit_message>
<xml_diff>
--- a/tabular/reference/herv_sublineage_data.xlsx
+++ b/tabular/reference/herv_sublineage_data.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A22FB3-E77A-A14B-A2C4-2A998CC7099D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D205A717-8EE7-B945-AB62-E252EA7B2FF3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1680" yWindow="520" windowWidth="27120" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1680" yWindow="520" windowWidth="27120" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sublineage" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="255">
   <si>
     <t>sequenceID</t>
   </si>
@@ -761,6 +762,30 @@
   </si>
   <si>
     <t>retinoic acid-responsive human endogenous retrovirus I</t>
+  </si>
+  <si>
+    <t>HERV-K-HML6-1a</t>
+  </si>
+  <si>
+    <t>HERV-K-HML6-1b</t>
+  </si>
+  <si>
+    <t>ERV-2.Beta.K6</t>
+  </si>
+  <si>
+    <t>HERV-K-HML6</t>
+  </si>
+  <si>
+    <t>endogenous archeobetaretrovirus K Catarrhini type 6</t>
+  </si>
+  <si>
+    <t>lineage</t>
+  </si>
+  <si>
+    <t>Archaeobetaretrovirus kappacatarrhini6</t>
+  </si>
+  <si>
+    <t>Archaeobeta</t>
   </si>
 </sst>
 </file>
@@ -6412,4 +6437,273 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E84FD6B7-DAC0-EF4A-B6E8-A6FD2C634E5A}">
+  <dimension ref="A1:Z3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="21.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2">
+        <v>8214</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="T2" s="2">
+        <v>20</v>
+      </c>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2">
+        <v>31167914</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z2" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2">
+        <v>8214</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="T3" s="2">
+        <v>20</v>
+      </c>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2">
+        <v>31167914</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="Z2">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z3">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z1">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Created build process for Homo sapiens ERV sublineage layer
</commit_message>
<xml_diff>
--- a/tabular/reference/herv_sublineage_data.xlsx
+++ b/tabular/reference/herv_sublineage_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D205A717-8EE7-B945-AB62-E252EA7B2FF3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF22DFF-BEF6-1E4D-B5EB-62CA9800B731}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1680" yWindow="520" windowWidth="27120" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1680" yWindow="1120" windowWidth="27120" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sublineage" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="256">
   <si>
     <t>sequenceID</t>
   </si>
@@ -779,13 +779,16 @@
     <t>endogenous archeobetaretrovirus K Catarrhini type 6</t>
   </si>
   <si>
-    <t>lineage</t>
-  </si>
-  <si>
-    <t>Archaeobetaretrovirus kappacatarrhini6</t>
-  </si>
-  <si>
     <t>Archaeobeta</t>
+  </si>
+  <si>
+    <t>lineage_id</t>
+  </si>
+  <si>
+    <t>ERV-2.Beta.K6.1a</t>
+  </si>
+  <si>
+    <t>ERV-2.Beta.K6.1b</t>
   </si>
 </sst>
 </file>
@@ -1687,7 +1690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB9083D8-DE01-F14E-ACB5-AF33867092C5}">
-  <dimension ref="A1:Z62"/>
+  <dimension ref="A1:Z57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.33203125" customWidth="1"/>
@@ -1710,7 +1713,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>169</v>
+        <v>253</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>82</v>
@@ -5125,19 +5128,19 @@
     </row>
     <row r="48" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
-        <v>177</v>
+        <v>8</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>178</v>
+        <v>124</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>179</v>
+        <v>8</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>245</v>
@@ -5154,41 +5157,43 @@
       <c r="J48" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K48" s="2" t="s">
-        <v>177</v>
+      <c r="K48" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="L48" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="M48" s="2"/>
+      <c r="M48" s="2">
+        <v>7048</v>
+      </c>
       <c r="N48" s="8" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="O48" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P48" s="2" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="Q48" s="1" t="s">
-        <v>183</v>
+        <v>10</v>
       </c>
       <c r="R48" s="2" t="s">
-        <v>172</v>
+        <v>6</v>
       </c>
       <c r="S48" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="T48" s="2"/>
       <c r="U48" s="2"/>
       <c r="V48" s="2">
-        <v>28397686</v>
+        <v>7692084</v>
       </c>
       <c r="W48" s="2" t="s">
         <v>12</v>
       </c>
       <c r="X48" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Y48" s="2" t="s">
         <v>12</v>
@@ -5199,19 +5204,19 @@
     </row>
     <row r="49" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
-        <v>180</v>
+        <v>14</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>181</v>
+        <v>125</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>182</v>
+        <v>14</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>245</v>
@@ -5228,41 +5233,45 @@
       <c r="J49" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K49" s="2" t="s">
-        <v>180</v>
+      <c r="K49" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="L49" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="M49" s="2"/>
+      <c r="M49" s="2">
+        <v>6364</v>
+      </c>
       <c r="N49" s="8" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="O49" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P49" s="2" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="Q49" s="1" t="s">
-        <v>184</v>
+        <v>10</v>
       </c>
       <c r="R49" s="2" t="s">
-        <v>172</v>
+        <v>6</v>
       </c>
       <c r="S49" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="T49" s="2"/>
+      <c r="T49" s="2">
+        <v>7</v>
+      </c>
       <c r="U49" s="2"/>
       <c r="V49" s="2">
-        <v>28397686</v>
+        <v>19540319</v>
       </c>
       <c r="W49" s="2" t="s">
         <v>12</v>
       </c>
       <c r="X49" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Y49" s="2" t="s">
         <v>12</v>
@@ -5273,19 +5282,19 @@
     </row>
     <row r="50" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
-        <v>185</v>
+        <v>15</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>186</v>
+        <v>126</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>187</v>
+        <v>15</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>245</v>
@@ -5302,41 +5311,45 @@
       <c r="J50" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K50" s="2" t="s">
-        <v>185</v>
+      <c r="K50" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="L50" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="M50" s="2"/>
+      <c r="M50" s="2">
+        <v>9472</v>
+      </c>
       <c r="N50" s="8" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="O50" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P50" s="2" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="Q50" s="1" t="s">
-        <v>188</v>
+        <v>10</v>
       </c>
       <c r="R50" s="2" t="s">
-        <v>172</v>
+        <v>6</v>
       </c>
       <c r="S50" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="T50" s="2"/>
+      <c r="T50" s="2">
+        <v>47</v>
+      </c>
       <c r="U50" s="2"/>
       <c r="V50" s="2">
-        <v>28397686</v>
+        <v>7692084</v>
       </c>
       <c r="W50" s="2" t="s">
         <v>12</v>
       </c>
       <c r="X50" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="Y50" s="2" t="s">
         <v>12</v>
@@ -5347,19 +5360,19 @@
     </row>
     <row r="51" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
-        <v>170</v>
+        <v>17</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>171</v>
+        <v>127</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>176</v>
+        <v>17</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>245</v>
@@ -5376,35 +5389,37 @@
       <c r="J51" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K51" s="2" t="s">
-        <v>170</v>
+      <c r="K51" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="L51" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="M51" s="2"/>
+      <c r="M51" s="2">
+        <v>7045</v>
+      </c>
       <c r="N51" s="8" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="O51" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P51" s="2" t="s">
-        <v>66</v>
+        <v>9</v>
       </c>
       <c r="Q51" s="1" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="R51" s="2" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="S51" s="2" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="T51" s="2"/>
       <c r="U51" s="2"/>
       <c r="V51" s="2">
-        <v>26952212</v>
+        <v>7692084</v>
       </c>
       <c r="W51" s="2" t="s">
         <v>12</v>
@@ -5413,27 +5428,27 @@
         <v>13</v>
       </c>
       <c r="Y51" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Z51" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
-        <v>173</v>
+        <v>18</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>174</v>
+        <v>128</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>175</v>
+        <v>18</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>104</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>245</v>
@@ -5450,58 +5465,62 @@
       <c r="J52" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K52" s="2" t="s">
-        <v>173</v>
+      <c r="K52" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="L52" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="M52" s="2"/>
+      <c r="M52" s="2">
+        <v>10243</v>
+      </c>
       <c r="N52" s="8" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="O52" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P52" s="2" t="s">
-        <v>66</v>
+        <v>9</v>
       </c>
       <c r="Q52" s="1" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="R52" s="2" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="S52" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="T52" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="T52" s="2">
+        <v>7</v>
+      </c>
       <c r="U52" s="2"/>
       <c r="V52" s="2">
-        <v>26952212</v>
+        <v>7692084</v>
       </c>
       <c r="W52" s="2" t="s">
         <v>12</v>
       </c>
       <c r="X52" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Y52" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Z52" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>104</v>
@@ -5531,7 +5550,7 @@
         <v>3</v>
       </c>
       <c r="M53" s="2">
-        <v>7048</v>
+        <v>8355</v>
       </c>
       <c r="N53" s="8" t="s">
         <v>4</v>
@@ -5549,12 +5568,14 @@
         <v>6</v>
       </c>
       <c r="S53" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="T53" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="T53" s="2">
+        <v>25</v>
+      </c>
       <c r="U53" s="2"/>
       <c r="V53" s="2">
-        <v>7692084</v>
+        <v>9934709</v>
       </c>
       <c r="W53" s="2" t="s">
         <v>12</v>
@@ -5571,13 +5592,13 @@
     </row>
     <row r="54" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A54" s="5" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>104</v>
@@ -5607,7 +5628,7 @@
         <v>3</v>
       </c>
       <c r="M54" s="2">
-        <v>6364</v>
+        <v>7274</v>
       </c>
       <c r="N54" s="8" t="s">
         <v>4</v>
@@ -5628,11 +5649,11 @@
         <v>7</v>
       </c>
       <c r="T54" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="U54" s="2"/>
       <c r="V54" s="2">
-        <v>19540319</v>
+        <v>9934709</v>
       </c>
       <c r="W54" s="2" t="s">
         <v>12</v>
@@ -5649,13 +5670,13 @@
     </row>
     <row r="55" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A55" s="5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>104</v>
@@ -5685,7 +5706,7 @@
         <v>3</v>
       </c>
       <c r="M55" s="2">
-        <v>9472</v>
+        <v>8214</v>
       </c>
       <c r="N55" s="8" t="s">
         <v>4</v>
@@ -5706,17 +5727,17 @@
         <v>7</v>
       </c>
       <c r="T55" s="2">
-        <v>47</v>
+        <v>104</v>
       </c>
       <c r="U55" s="2"/>
       <c r="V55" s="2">
-        <v>7692084</v>
+        <v>19540319</v>
       </c>
       <c r="W55" s="2" t="s">
         <v>12</v>
       </c>
       <c r="X55" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="Y55" s="2" t="s">
         <v>12</v>
@@ -5727,19 +5748,19 @@
     </row>
     <row r="56" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A56" s="5" t="s">
-        <v>17</v>
+        <v>97</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>17</v>
+        <v>97</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>245</v>
@@ -5748,34 +5769,34 @@
         <v>121</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>13</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="L56" s="2" t="s">
         <v>3</v>
       </c>
       <c r="M56" s="2">
-        <v>7045</v>
+        <v>6896</v>
       </c>
       <c r="N56" s="8" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="O56" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P56" s="2" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="Q56" s="1" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="R56" s="2" t="s">
         <v>6</v>
@@ -5785,9 +5806,7 @@
       </c>
       <c r="T56" s="2"/>
       <c r="U56" s="2"/>
-      <c r="V56" s="2">
-        <v>7692084</v>
-      </c>
+      <c r="V56" s="2"/>
       <c r="W56" s="2" t="s">
         <v>12</v>
       </c>
@@ -5795,27 +5814,27 @@
         <v>13</v>
       </c>
       <c r="Y56" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Z56" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A57" s="5" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>245</v>
@@ -5824,450 +5843,64 @@
         <v>121</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>13</v>
+        <v>219</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K57" s="1" t="s">
-        <v>98</v>
+        <v>16</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="L57" s="2" t="s">
         <v>3</v>
       </c>
       <c r="M57" s="2">
-        <v>10243</v>
+        <v>5685</v>
       </c>
       <c r="N57" s="8" t="s">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="O57" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P57" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q57" s="1" t="s">
-        <v>10</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="Q57" s="1"/>
       <c r="R57" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="S57" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="T57" s="2">
-        <v>7</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="T57" s="2"/>
       <c r="U57" s="2"/>
-      <c r="V57" s="2">
-        <v>7692084</v>
-      </c>
+      <c r="V57" s="2"/>
       <c r="W57" s="2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="X57" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Y57" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Z57" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A58" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H58" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J58" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K58" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="L58" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="M58" s="2">
-        <v>8355</v>
-      </c>
-      <c r="N58" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="O58" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="P58" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q58" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="R58" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="S58" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="T58" s="2">
-        <v>25</v>
-      </c>
-      <c r="U58" s="2"/>
-      <c r="V58" s="2">
-        <v>9934709</v>
-      </c>
-      <c r="W58" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X58" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y58" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z58" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A59" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H59" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="I59" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J59" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K59" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="L59" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="M59" s="2">
-        <v>7274</v>
-      </c>
-      <c r="N59" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="O59" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="P59" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q59" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="R59" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="S59" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="T59" s="2">
-        <v>10</v>
-      </c>
-      <c r="U59" s="2"/>
-      <c r="V59" s="2">
-        <v>9934709</v>
-      </c>
-      <c r="W59" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X59" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y59" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z59" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A60" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K60" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="L60" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="M60" s="2">
-        <v>8214</v>
-      </c>
-      <c r="N60" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="O60" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="P60" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q60" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="R60" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="S60" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="T60" s="2">
-        <v>104</v>
-      </c>
-      <c r="U60" s="2"/>
-      <c r="V60" s="2">
-        <v>19540319</v>
-      </c>
-      <c r="W60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X60" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y60" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z60" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A61" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="G61" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="I61" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J61" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K61" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="L61" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="M61" s="2">
-        <v>6896</v>
-      </c>
-      <c r="N61" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="O61" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="P61" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q61" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="R61" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="S61" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="T61" s="2"/>
-      <c r="U61" s="2"/>
-      <c r="V61" s="2"/>
-      <c r="W61" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X61" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y61" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z61" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A62" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="G62" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H62" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="I62" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="J62" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K62" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="L62" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="M62" s="2">
-        <v>5685</v>
-      </c>
-      <c r="N62" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="O62" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="P62" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q62" s="1"/>
-      <c r="R62" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S62" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="T62" s="2"/>
-      <c r="U62" s="2"/>
-      <c r="V62" s="2"/>
-      <c r="W62" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="X62" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y62" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z62" s="2">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z62">
-    <sortCondition ref="G2:G62"/>
-    <sortCondition ref="H2:H62"/>
-    <sortCondition ref="N2:N62"/>
-    <sortCondition ref="P2:P62"/>
-    <sortCondition ref="Q2:Q62"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z57">
+    <sortCondition ref="G2:G57"/>
+    <sortCondition ref="H2:H57"/>
+    <sortCondition ref="N2:N57"/>
+    <sortCondition ref="P2:P57"/>
+    <sortCondition ref="Q2:Q57"/>
   </sortState>
-  <conditionalFormatting sqref="Z63:Z1048576 Z1:Z45">
+  <conditionalFormatting sqref="Z58:Z1048576 Z1:Z45">
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
@@ -6279,7 +5912,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z46:Z49">
+  <conditionalFormatting sqref="Z46:Z47">
     <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
@@ -6291,8 +5924,92 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z50:Z51">
-    <cfRule type="colorScale" priority="18">
+  <conditionalFormatting sqref="Z48">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z49">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z50">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z51">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z54">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z55">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z56">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z57">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -6304,7 +6021,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z52">
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -6316,114 +6033,6 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z53">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z54">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z55">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z56">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z59">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z60">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z61">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z62">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z57">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z58">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6441,10 +6050,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E84FD6B7-DAC0-EF4A-B6E8-A6FD2C634E5A}">
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="4" max="4" width="40.5" customWidth="1"/>
+    <col min="5" max="5" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.2">
@@ -6532,7 +6144,7 @@
         <v>247</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>250</v>
@@ -6541,13 +6153,13 @@
         <v>251</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>253</v>
+        <v>249</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>3</v>
+        <v>121</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
@@ -6569,7 +6181,7 @@
         <v>9</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>6</v>
@@ -6602,7 +6214,7 @@
         <v>248</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>250</v>
@@ -6611,13 +6223,13 @@
         <v>251</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>253</v>
+        <v>249</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>3</v>
+        <v>121</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
@@ -6639,7 +6251,7 @@
         <v>9</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>6</v>
@@ -6667,8 +6279,426 @@
         <v>1</v>
       </c>
     </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4" s="2"/>
+      <c r="N4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2">
+        <v>28397686</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" s="2"/>
+      <c r="N5" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2">
+        <v>28397686</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z5" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M6" s="2"/>
+      <c r="N6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2">
+        <v>28397686</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z6" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M7" s="2"/>
+      <c r="N7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2">
+        <v>26952212</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z7" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M8" s="2"/>
+      <c r="N8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2">
+        <v>26952212</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z8" s="2">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="Z2">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z3">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z1">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z4:Z5">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z6:Z7">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -6680,20 +6710,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z3">
+  <conditionalFormatting sqref="Z8">
     <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z1">
-    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>